<commit_message>
Update tour spreadsheet with new file (adds a Mexico-only summary tab)
New version adds a dedicated "MEXICO" sheet alongside the original
"WORLD TOUR 2027" sheet. Totals and city-by-city data in the main
sheet are unchanged (80,350 attendees, 92 cities), so no content on
the page needed updating — just the linked file.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/tour-2027-numbers.xlsx
+++ b/assets/tour-2027-numbers.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/regulocastrogomez/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86321418-ED0D-7648-A2A6-C757493927C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC7E706-258F-3D49-A496-6DC6E358F37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" xr2:uid="{BBF3B1B2-2BD0-D242-B940-7BB9A5C7F668}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{BBF3B1B2-2BD0-D242-B940-7BB9A5C7F668}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="WORLD TOUR 2027" sheetId="1" r:id="rId1"/>
+    <sheet name="MEXICO" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="105">
   <si>
     <t>CD. JUAREZ</t>
   </si>
@@ -351,6 +352,9 @@
   </si>
   <si>
     <t>AUGUST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHIAPAS </t>
   </si>
 </sst>
 </file>
@@ -545,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -631,6 +635,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -974,6 +981,10 @@
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="23.33203125" customWidth="1"/>
+    <col min="10" max="10" width="12.5" customWidth="1"/>
+    <col min="11" max="11" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3221,4 +3232,651 @@
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CAEE08B-A1D7-8A4E-9058-11073D6B376D}">
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="21.1640625" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" customWidth="1"/>
+    <col min="3" max="3" width="29.5" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="22">
+      <c r="A1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="20">
+      <c r="A2" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="17"/>
+    </row>
+    <row r="3" spans="1:4" ht="20">
+      <c r="A3" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C3" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4" ht="20">
+      <c r="A4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C4" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D4" s="17"/>
+    </row>
+    <row r="5" spans="1:4" ht="20">
+      <c r="A5" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C5" s="10">
+        <v>17500</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="20">
+      <c r="A6" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C6" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D6" s="17"/>
+    </row>
+    <row r="7" spans="1:4" ht="22">
+      <c r="A7" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1000</v>
+      </c>
+      <c r="C7" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D7" s="27"/>
+    </row>
+    <row r="8" spans="1:4" ht="20">
+      <c r="A8" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1000</v>
+      </c>
+      <c r="C8" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D8" s="16"/>
+    </row>
+    <row r="9" spans="1:4" ht="20">
+      <c r="A9" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C9" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D9" s="16"/>
+    </row>
+    <row r="10" spans="1:4" ht="20">
+      <c r="D10" s="26">
+        <f>SUM(C3:C9)</f>
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="20">
+      <c r="A11" s="11"/>
+      <c r="B11" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="20">
+      <c r="A12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="2">
+        <v>600</v>
+      </c>
+      <c r="C12" s="15">
+        <v>5250</v>
+      </c>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:4" ht="20">
+      <c r="A13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="2">
+        <v>600</v>
+      </c>
+      <c r="C13" s="15">
+        <v>5250</v>
+      </c>
+      <c r="D13" s="17"/>
+    </row>
+    <row r="14" spans="1:4" ht="20">
+      <c r="A14" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="2">
+        <v>800</v>
+      </c>
+      <c r="C14" s="15">
+        <v>7000</v>
+      </c>
+      <c r="D14" s="17"/>
+    </row>
+    <row r="15" spans="1:4" ht="20">
+      <c r="A15" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C15" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D15" s="17"/>
+    </row>
+    <row r="16" spans="1:4" ht="20">
+      <c r="A16" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C16" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D16" s="17"/>
+    </row>
+    <row r="17" spans="1:4" ht="20">
+      <c r="D17" s="26">
+        <f>SUM(C12:C16)</f>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="20">
+      <c r="A18" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="13">
+        <v>1300</v>
+      </c>
+      <c r="C18" s="10">
+        <v>11375</v>
+      </c>
+      <c r="D18" s="17"/>
+    </row>
+    <row r="19" spans="1:4" ht="20">
+      <c r="A19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="13">
+        <v>1500</v>
+      </c>
+      <c r="C19" s="10">
+        <v>13125</v>
+      </c>
+      <c r="D19" s="17"/>
+    </row>
+    <row r="20" spans="1:4" ht="20">
+      <c r="A20" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="13">
+        <v>1700</v>
+      </c>
+      <c r="C20" s="10">
+        <v>14875</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="22">
+      <c r="A21" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C21" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D21" s="27"/>
+    </row>
+    <row r="23" spans="1:4" ht="22">
+      <c r="A23" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="27"/>
+    </row>
+    <row r="24" spans="1:4" ht="20">
+      <c r="A24" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C24" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D24" s="17"/>
+    </row>
+    <row r="25" spans="1:4" ht="20">
+      <c r="A25" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C25" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D25" s="17"/>
+    </row>
+    <row r="26" spans="1:4" ht="20">
+      <c r="A26" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C26" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D26" s="17"/>
+    </row>
+    <row r="27" spans="1:4" ht="20">
+      <c r="A27" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C27" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D27" s="17"/>
+    </row>
+    <row r="28" spans="1:4" ht="20">
+      <c r="A28" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C28" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D28" s="17"/>
+    </row>
+    <row r="29" spans="1:4" ht="20">
+      <c r="A29" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B29" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C29" s="10">
+        <v>15000</v>
+      </c>
+      <c r="D29" s="26">
+        <f>SUM(C24:C28)</f>
+        <v>43750</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="22">
+      <c r="A31" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="D31" s="27"/>
+    </row>
+    <row r="32" spans="1:4" ht="22">
+      <c r="A32" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C32" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D32" s="27"/>
+    </row>
+    <row r="33" spans="1:4" ht="20">
+      <c r="A33" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C33" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D33" s="17"/>
+    </row>
+    <row r="34" spans="1:4" ht="20">
+      <c r="A34" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C34" s="10">
+        <v>17500</v>
+      </c>
+      <c r="D34" s="17"/>
+    </row>
+    <row r="35" spans="1:4" ht="20">
+      <c r="A35" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C35" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D35" s="17"/>
+    </row>
+    <row r="36" spans="1:4" ht="20">
+      <c r="A36" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C36" s="15">
+        <v>8750</v>
+      </c>
+      <c r="D36" s="17"/>
+    </row>
+    <row r="37" spans="1:4" ht="22">
+      <c r="A37" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C37" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D37" s="27"/>
+    </row>
+    <row r="38" spans="1:4" ht="20">
+      <c r="A38" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C38" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D38" s="17"/>
+    </row>
+    <row r="39" spans="1:4" ht="20">
+      <c r="A39" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B39" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C39" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D39" s="17"/>
+    </row>
+    <row r="40" spans="1:4" ht="20">
+      <c r="A40" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="26">
+        <f>SUM(C32:C39)</f>
+        <v>78750</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="20">
+      <c r="A41" s="9"/>
+      <c r="B41" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="C41" s="9"/>
+      <c r="D41" s="17"/>
+    </row>
+    <row r="42" spans="1:4" ht="20">
+      <c r="A42" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="13">
+        <v>1500</v>
+      </c>
+      <c r="C42" s="10">
+        <v>13125</v>
+      </c>
+      <c r="D42" s="17"/>
+    </row>
+    <row r="43" spans="1:4" ht="20">
+      <c r="A43" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B43" s="13">
+        <v>1700</v>
+      </c>
+      <c r="C43" s="10">
+        <v>14875</v>
+      </c>
+      <c r="D43" s="17"/>
+    </row>
+    <row r="44" spans="1:4" ht="20">
+      <c r="A44" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" s="3">
+        <v>1500</v>
+      </c>
+      <c r="C44" s="10">
+        <v>13125</v>
+      </c>
+      <c r="D44" s="17"/>
+    </row>
+    <row r="45" spans="1:4" ht="20">
+      <c r="A45" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="3">
+        <v>1000</v>
+      </c>
+      <c r="C45" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D45" s="17"/>
+    </row>
+    <row r="46" spans="1:4" ht="20">
+      <c r="A46" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B46" s="3">
+        <v>1500</v>
+      </c>
+      <c r="C46" s="10">
+        <v>13125</v>
+      </c>
+      <c r="D46" s="17"/>
+    </row>
+    <row r="47" spans="1:4" ht="22">
+      <c r="A47" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B47" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C47" s="10">
+        <v>17000</v>
+      </c>
+      <c r="D47" s="27"/>
+    </row>
+    <row r="48" spans="1:4" ht="22">
+      <c r="A48" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B48" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C48" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D48" s="27"/>
+    </row>
+    <row r="49" spans="1:4" ht="22">
+      <c r="D49" s="35">
+        <f>SUM(C42:C48)</f>
+        <v>88750</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="22">
+      <c r="A51" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B51" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C51" s="12"/>
+      <c r="D51" s="28"/>
+    </row>
+    <row r="52" spans="1:4" ht="20">
+      <c r="A52" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C52" s="10">
+        <v>17500</v>
+      </c>
+      <c r="D52" s="28"/>
+    </row>
+    <row r="53" spans="1:4" ht="20">
+      <c r="A53" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B53" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C53" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D53" s="28"/>
+    </row>
+    <row r="54" spans="1:4" ht="20">
+      <c r="A54" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" s="13">
+        <v>1000</v>
+      </c>
+      <c r="C54" s="10">
+        <v>8750</v>
+      </c>
+      <c r="D54" s="28"/>
+    </row>
+    <row r="55" spans="1:4" ht="20">
+      <c r="A55" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B55" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C55" s="10">
+        <v>17500</v>
+      </c>
+      <c r="D55" s="28"/>
+    </row>
+    <row r="56" spans="1:4" ht="20">
+      <c r="A56" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C56" s="10">
+        <v>17500</v>
+      </c>
+      <c r="D56" s="28"/>
+    </row>
+    <row r="57" spans="1:4" ht="20">
+      <c r="A57" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="13">
+        <v>2000</v>
+      </c>
+      <c r="C57" s="10">
+        <v>17500</v>
+      </c>
+      <c r="D57" s="28"/>
+    </row>
+    <row r="58" spans="1:4" ht="20">
+      <c r="B58" s="9"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="26">
+        <f>SUM(C52:C58)</f>
+        <v>87500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>